<commit_message>
add 6 dimension pedsQL
</commit_message>
<xml_diff>
--- a/data/Marfan.xlsx
+++ b/data/Marfan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chloe/Documents/Laignel.Chloe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57291AAD-A724-D845-B874-409C04F3B853}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FCE054-3705-D249-B68F-F21B1ED4373A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="20">
   <si>
     <t>ID</t>
   </si>
@@ -67,6 +67,24 @@
   </si>
   <si>
     <t>PEDSQL_totalself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_santeself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_emotionself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_relationself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_ecoleself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_psycosocialself_after</t>
+  </si>
+  <si>
+    <t>PEDSQL_physiqueself_after</t>
   </si>
 </sst>
 </file>
@@ -111,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -147,11 +165,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -206,6 +242,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -488,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="27.6640625" customWidth="1"/>
@@ -500,9 +548,15 @@
     <col min="10" max="10" width="27.83203125" customWidth="1"/>
     <col min="11" max="11" width="20.1640625" customWidth="1"/>
     <col min="12" max="12" width="21.1640625" customWidth="1"/>
+    <col min="13" max="13" width="24.5" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="21.1640625" customWidth="1"/>
+    <col min="16" max="16" width="25.33203125" customWidth="1"/>
+    <col min="17" max="17" width="26.33203125" customWidth="1"/>
+    <col min="18" max="18" width="25.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -539,8 +593,26 @@
       <c r="L1" s="18" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M1" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="P1" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q1" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="R1" s="18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -577,8 +649,26 @@
       <c r="L2" s="16">
         <v>75</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M2" s="20">
+        <v>71.875</v>
+      </c>
+      <c r="N2" s="20">
+        <v>70</v>
+      </c>
+      <c r="O2" s="20">
+        <v>85</v>
+      </c>
+      <c r="P2" s="20">
+        <v>75</v>
+      </c>
+      <c r="Q2" s="20">
+        <v>76.666666666666671</v>
+      </c>
+      <c r="R2" s="20">
+        <v>71.875</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -609,8 +699,14 @@
         <v>86.956521739130437</v>
       </c>
       <c r="L3" s="19"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
         <v>3</v>
       </c>
@@ -647,8 +743,26 @@
       <c r="L4" s="19">
         <v>92.391304347826093</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M4" s="23">
+        <v>96.875</v>
+      </c>
+      <c r="N4" s="23">
+        <v>85</v>
+      </c>
+      <c r="O4" s="23">
+        <v>100</v>
+      </c>
+      <c r="P4" s="23">
+        <v>85</v>
+      </c>
+      <c r="Q4" s="23">
+        <v>90</v>
+      </c>
+      <c r="R4" s="23">
+        <v>96.875</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -685,8 +799,26 @@
       <c r="L5" s="16">
         <v>57.608695652173914</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M5" s="21">
+        <v>53.125</v>
+      </c>
+      <c r="N5" s="21">
+        <v>55</v>
+      </c>
+      <c r="O5" s="21">
+        <v>55</v>
+      </c>
+      <c r="P5" s="21">
+        <v>70</v>
+      </c>
+      <c r="Q5" s="21">
+        <v>60</v>
+      </c>
+      <c r="R5" s="21">
+        <v>53.125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
         <v>5</v>
       </c>
@@ -719,8 +851,26 @@
       <c r="L6" s="19">
         <v>70.652173913043484</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M6" s="23">
+        <v>53.125</v>
+      </c>
+      <c r="N6" s="23">
+        <v>65</v>
+      </c>
+      <c r="O6" s="23">
+        <v>75</v>
+      </c>
+      <c r="P6" s="23">
+        <v>100</v>
+      </c>
+      <c r="Q6" s="23">
+        <v>80</v>
+      </c>
+      <c r="R6" s="23">
+        <v>53.125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -757,8 +907,26 @@
       <c r="L7" s="16">
         <v>95.652173913043484</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M7" s="21">
+        <v>100</v>
+      </c>
+      <c r="N7" s="21">
+        <v>90</v>
+      </c>
+      <c r="O7" s="21">
+        <v>100</v>
+      </c>
+      <c r="P7" s="21">
+        <v>90</v>
+      </c>
+      <c r="Q7" s="21">
+        <v>93.333333333333329</v>
+      </c>
+      <c r="R7" s="21">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
         <v>7</v>
       </c>
@@ -789,8 +957,14 @@
         <v>75</v>
       </c>
       <c r="L8" s="19"/>
-    </row>
-    <row r="9" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+    </row>
+    <row r="9" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -827,8 +1001,26 @@
       <c r="L9" s="16">
         <v>82.608695652173907</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M9" s="21">
+        <v>100</v>
+      </c>
+      <c r="N9" s="21">
+        <v>75</v>
+      </c>
+      <c r="O9" s="21">
+        <v>85</v>
+      </c>
+      <c r="P9" s="21">
+        <v>60</v>
+      </c>
+      <c r="Q9" s="21">
+        <v>73.333333333333329</v>
+      </c>
+      <c r="R9" s="21">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -865,8 +1057,26 @@
       <c r="L10" s="16">
         <v>88.043478260869563</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M10" s="21">
+        <v>90.625</v>
+      </c>
+      <c r="N10" s="21">
+        <v>85</v>
+      </c>
+      <c r="O10" s="21">
+        <v>90</v>
+      </c>
+      <c r="P10" s="21">
+        <v>85</v>
+      </c>
+      <c r="Q10" s="21">
+        <v>86.666666666666671</v>
+      </c>
+      <c r="R10" s="21">
+        <v>90.625</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -903,8 +1113,26 @@
       <c r="L11" s="16">
         <v>97.826086956521735</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M11" s="21">
+        <v>96.875</v>
+      </c>
+      <c r="N11" s="21">
+        <v>100</v>
+      </c>
+      <c r="O11" s="21">
+        <v>100</v>
+      </c>
+      <c r="P11" s="21">
+        <v>95</v>
+      </c>
+      <c r="Q11" s="21">
+        <v>98.333333333333329</v>
+      </c>
+      <c r="R11" s="21">
+        <v>96.875</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -941,8 +1169,26 @@
       <c r="L12" s="16">
         <v>92.391304347826093</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M12" s="21">
+        <v>90.625</v>
+      </c>
+      <c r="N12" s="21">
+        <v>95</v>
+      </c>
+      <c r="O12" s="21">
+        <v>100</v>
+      </c>
+      <c r="P12" s="21">
+        <v>85</v>
+      </c>
+      <c r="Q12" s="21">
+        <v>93.333333333333329</v>
+      </c>
+      <c r="R12" s="21">
+        <v>90.625</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
         <v>12</v>
       </c>
@@ -975,8 +1221,26 @@
       <c r="L13" s="19">
         <v>75</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M13" s="23">
+        <v>78.125</v>
+      </c>
+      <c r="N13" s="23">
+        <v>65</v>
+      </c>
+      <c r="O13" s="23">
+        <v>75</v>
+      </c>
+      <c r="P13" s="23">
+        <v>80</v>
+      </c>
+      <c r="Q13" s="23">
+        <v>73.333333333333329</v>
+      </c>
+      <c r="R13" s="23">
+        <v>78.125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1013,8 +1277,26 @@
       <c r="L14" s="16">
         <v>73.913043478260875</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M14" s="21">
+        <v>65.625</v>
+      </c>
+      <c r="N14" s="21">
+        <v>85</v>
+      </c>
+      <c r="O14" s="21">
+        <v>75</v>
+      </c>
+      <c r="P14" s="21">
+        <v>75</v>
+      </c>
+      <c r="Q14" s="21">
+        <v>78.333333333333329</v>
+      </c>
+      <c r="R14" s="21">
+        <v>65.625</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1051,8 +1333,26 @@
       <c r="L15" s="16">
         <v>72.826086956521735</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M15" s="21">
+        <v>90.625</v>
+      </c>
+      <c r="N15" s="21">
+        <v>60</v>
+      </c>
+      <c r="O15" s="21">
+        <v>80</v>
+      </c>
+      <c r="P15" s="21">
+        <v>50</v>
+      </c>
+      <c r="Q15" s="21">
+        <v>63.333333333333336</v>
+      </c>
+      <c r="R15" s="21">
+        <v>90.625</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1089,8 +1389,26 @@
       <c r="L16" s="16">
         <v>86.956521739130437</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M16" s="21">
+        <v>87.5</v>
+      </c>
+      <c r="N16" s="21">
+        <v>90</v>
+      </c>
+      <c r="O16" s="21">
+        <v>90</v>
+      </c>
+      <c r="P16" s="21">
+        <v>80</v>
+      </c>
+      <c r="Q16" s="21">
+        <v>86.666666666666671</v>
+      </c>
+      <c r="R16" s="21">
+        <v>87.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -1121,8 +1439,14 @@
         <v>83.695652173913047</v>
       </c>
       <c r="L17" s="19"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="19"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -1153,8 +1477,14 @@
         <v>46.739130434782609</v>
       </c>
       <c r="L18" s="19"/>
-    </row>
-    <row r="19" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="19"/>
+      <c r="Q18" s="19"/>
+      <c r="R18" s="19"/>
+    </row>
+    <row r="19" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1191,8 +1521,26 @@
       <c r="L19" s="16">
         <v>77.173913043478265</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M19" s="21">
+        <v>62.5</v>
+      </c>
+      <c r="N19" s="21">
+        <v>90</v>
+      </c>
+      <c r="O19" s="21">
+        <v>80</v>
+      </c>
+      <c r="P19" s="21">
+        <v>85</v>
+      </c>
+      <c r="Q19" s="21">
+        <v>85</v>
+      </c>
+      <c r="R19" s="21">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1229,8 +1577,26 @@
       <c r="L20" s="16">
         <v>89.130434782608702</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M20" s="21">
+        <v>93.75</v>
+      </c>
+      <c r="N20" s="21">
+        <v>100</v>
+      </c>
+      <c r="O20" s="21">
+        <v>80</v>
+      </c>
+      <c r="P20" s="21">
+        <v>80</v>
+      </c>
+      <c r="Q20" s="21">
+        <v>86.666666666666671</v>
+      </c>
+      <c r="R20" s="21">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1267,8 +1633,26 @@
       <c r="L21" s="16">
         <v>64.130434782608702</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M21" s="21">
+        <v>75</v>
+      </c>
+      <c r="N21" s="21">
+        <v>40</v>
+      </c>
+      <c r="O21" s="21">
+        <v>80</v>
+      </c>
+      <c r="P21" s="21">
+        <v>55</v>
+      </c>
+      <c r="Q21" s="21">
+        <v>58.333333333333336</v>
+      </c>
+      <c r="R21" s="21">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1305,8 +1689,26 @@
       <c r="L22" s="16">
         <v>83.695652173913047</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M22" s="21">
+        <v>90.625</v>
+      </c>
+      <c r="N22" s="21">
+        <v>80</v>
+      </c>
+      <c r="O22" s="21">
+        <v>100</v>
+      </c>
+      <c r="P22" s="21">
+        <v>60</v>
+      </c>
+      <c r="Q22" s="21">
+        <v>80</v>
+      </c>
+      <c r="R22" s="21">
+        <v>90.625</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1343,8 +1745,26 @@
       <c r="L23" s="16">
         <v>71.739130434782609</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M23" s="21">
+        <v>71.875</v>
+      </c>
+      <c r="N23" s="21">
+        <v>75</v>
+      </c>
+      <c r="O23" s="21">
+        <v>70</v>
+      </c>
+      <c r="P23" s="21">
+        <v>70</v>
+      </c>
+      <c r="Q23" s="21">
+        <v>71.666666666666671</v>
+      </c>
+      <c r="R23" s="21">
+        <v>71.875</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1381,8 +1801,26 @@
       <c r="L24" s="16">
         <v>70.652173913043484</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M24" s="21">
+        <v>62.5</v>
+      </c>
+      <c r="N24" s="21">
+        <v>70</v>
+      </c>
+      <c r="O24" s="21">
+        <v>80</v>
+      </c>
+      <c r="P24" s="21">
+        <v>75</v>
+      </c>
+      <c r="Q24" s="21">
+        <v>75</v>
+      </c>
+      <c r="R24" s="21">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1419,8 +1857,26 @@
       <c r="L25" s="16">
         <v>78.260869565217391</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25" s="21">
+        <v>93.75</v>
+      </c>
+      <c r="N25" s="21">
+        <v>70</v>
+      </c>
+      <c r="O25" s="21">
+        <v>100</v>
+      </c>
+      <c r="P25" s="21">
+        <v>40</v>
+      </c>
+      <c r="Q25" s="21">
+        <v>70</v>
+      </c>
+      <c r="R25" s="21">
+        <v>93.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -1451,8 +1907,14 @@
         <v>34.782608695652172</v>
       </c>
       <c r="L26" s="19"/>
-    </row>
-    <row r="27" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M26" s="19"/>
+      <c r="N26" s="19"/>
+      <c r="O26" s="19"/>
+      <c r="P26" s="19"/>
+      <c r="Q26" s="19"/>
+      <c r="R26" s="19"/>
+    </row>
+    <row r="27" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1489,8 +1951,26 @@
       <c r="L27" s="16">
         <v>59.782608695652172</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27" s="21">
+        <v>65.625</v>
+      </c>
+      <c r="N27" s="21">
+        <v>55</v>
+      </c>
+      <c r="O27" s="21">
+        <v>65</v>
+      </c>
+      <c r="P27" s="21">
+        <v>50</v>
+      </c>
+      <c r="Q27" s="21">
+        <v>56.666666666666664</v>
+      </c>
+      <c r="R27" s="21">
+        <v>65.625</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -1521,8 +2001,14 @@
         <v>46.739130434782609</v>
       </c>
       <c r="L28" s="19"/>
-    </row>
-    <row r="29" spans="1:12" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="19"/>
+    </row>
+    <row r="29" spans="1:18" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -1559,8 +2045,26 @@
       <c r="L29" s="16">
         <v>80.434782608695656</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" s="22">
+        <v>68.75</v>
+      </c>
+      <c r="N29" s="22">
+        <v>90</v>
+      </c>
+      <c r="O29" s="22">
+        <v>80</v>
+      </c>
+      <c r="P29" s="22">
+        <v>90</v>
+      </c>
+      <c r="Q29" s="22">
+        <v>86.666666666666671</v>
+      </c>
+      <c r="R29" s="22">
+        <v>68.75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="I30" s="6"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>